<commit_message>
chore: update Instagram report 2026-10-13 11:36
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/2026-10-13.xlsx
+++ b/instagram-daily-checker/reports/2026-10-13.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-13 11:17:09</t>
+          <t>取得日時：2026-10-13 11:36:02</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">

</xml_diff>